<commit_message>
docs(wbs): update completed work-package status
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{C84441A9-493A-415C-B430-AB0EFCA297E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FC79891-191C-458E-B238-2271FE52CAF7}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C84441A9-493A-415C-B430-AB0EFCA297E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7038D520-20FD-4BCA-A22B-CE50EC350255}"/>
   <bookViews>
-    <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14085" yWindow="-16200" windowWidth="29010" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -3831,7 +3831,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.24691358024691362</c:v>
+                  <c:v>0.37037037037037041</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4016,10 +4016,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4322,14 +4318,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.10463215258855582</v>
+        <v>0.11553133514986372</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>9.3732970027247925E-2</v>
+        <v>0.10463215258855582</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4346,7 +4342,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4451,11 +4447,11 @@
       </c>
       <c r="F13" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A13,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A13,WBS!$R$5:$R$137),0)</f>
-        <v>0.24691358024691362</v>
+        <v>0.37037037037037041</v>
       </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>0.24691358024691362</v>
+        <v>0.37037037037037041</v>
       </c>
       <c r="H13" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A13)</f>
@@ -4463,7 +4459,7 @@
       </c>
       <c r="I13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Complete")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Late")</f>
@@ -4951,7 +4947,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.10463215258855582</v>
+        <v>0.11553133514986372</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4966,7 +4962,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>9.3732970027247925E-2</v>
+        <v>0.10463215258855582</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4996,7 +4992,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6244,7 +6240,7 @@
         <v>0</v>
       </c>
       <c r="Q18" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R18" s="14">
         <f t="shared" si="0"/>
@@ -6256,11 +6252,11 @@
       </c>
       <c r="T18" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U18" t="str">
         <f>IF(Q18&gt;=1,"Complete",IF(Q18&gt;0,"In Progress",IF(Control!$B$7&lt;H18,"Not Started",IF(Control!$B$7&gt;I18,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V18" s="15">
         <v>46265</v>
@@ -6317,7 +6313,7 @@
         <v>0</v>
       </c>
       <c r="Q19" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" s="14">
         <f t="shared" si="0"/>
@@ -6329,11 +6325,11 @@
       </c>
       <c r="T19" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U19" t="str">
         <f>IF(Q19&gt;=1,"Complete",IF(Q19&gt;0,"In Progress",IF(Control!$B$7&lt;H19,"Not Started",IF(Control!$B$7&gt;I19,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V19" s="15">
         <v>46272</v>
@@ -15318,22 +15314,22 @@
       </c>
       <c r="H8" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A8,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A8,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I8" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="J8" s="4">
         <v>3</v>
       </c>
       <c r="K8" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A8,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="str">
         <f>IF(H8&gt;=1,"Complete",IF(H8&gt;0,"In Progress",IF(Control!$B$7&lt;D8,"Not Started",IF(Control!$B$7&gt;E8,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -16973,7 +16969,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.10463215258855582</v>
+        <v>0.11553133514986372</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>

<commit_message>
docs(wbs): update completed work-package status (#6)
</commit_message>
<xml_diff>
--- a/ESP32_S3_SQD_Project_WBS.xlsx
+++ b/ESP32_S3_SQD_Project_WBS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4f91d42a59b2d5e5/SQD/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="13_ncr:1_{C84441A9-493A-415C-B430-AB0EFCA297E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3FC79891-191C-458E-B238-2271FE52CAF7}"/>
+  <xr:revisionPtr revIDLastSave="33" documentId="13_ncr:1_{C84441A9-493A-415C-B430-AB0EFCA297E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7038D520-20FD-4BCA-A22B-CE50EC350255}"/>
   <bookViews>
-    <workbookView xWindow="-14730" yWindow="-16320" windowWidth="57840" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14085" yWindow="-16200" windowWidth="29010" windowHeight="15585" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -3831,7 +3831,7 @@
                   <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.24691358024691362</c:v>
+                  <c:v>0.37037037037037041</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -4016,10 +4016,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4322,14 +4318,14 @@
       </c>
       <c r="E5" s="12">
         <f>Control!B11</f>
-        <v>0.10463215258855582</v>
+        <v>0.11553133514986372</v>
       </c>
       <c r="G5" s="9" t="s">
         <v>6</v>
       </c>
       <c r="H5" s="12">
         <f>Control!B12</f>
-        <v>9.3732970027247925E-2</v>
+        <v>0.10463215258855582</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="30" customHeight="1"/>
@@ -4346,7 +4342,7 @@
       </c>
       <c r="E7" s="11">
         <f>Control!B14</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="G7" s="9" t="s">
         <v>9</v>
@@ -4451,11 +4447,11 @@
       </c>
       <c r="F13" s="6">
         <f>IFERROR(SUMIF(WBS!$B$5:$B$137,A13,WBS!$T$5:$T$137)/SUMIF(WBS!$B$5:$B$137,A13,WBS!$R$5:$R$137),0)</f>
-        <v>0.24691358024691362</v>
+        <v>0.37037037037037041</v>
       </c>
       <c r="G13" s="6">
         <f t="shared" si="0"/>
-        <v>0.24691358024691362</v>
+        <v>0.37037037037037041</v>
       </c>
       <c r="H13" s="4">
         <f>COUNTIF(WBS!$B$5:$B$137,A13)</f>
@@ -4463,7 +4459,7 @@
       </c>
       <c r="I13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Complete")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J13" s="4">
         <f>COUNTIFS(WBS!$B$5:$B$137,A13,WBS!$U$5:$U$137,"Late")</f>
@@ -4951,7 +4947,7 @@
       </c>
       <c r="B11" s="6">
         <f>SUM(WBS!T5:T137)</f>
-        <v>0.10463215258855582</v>
+        <v>0.11553133514986372</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>69</v>
@@ -4966,7 +4962,7 @@
       </c>
       <c r="B12" s="6">
         <f>B11-B10</f>
-        <v>9.3732970027247925E-2</v>
+        <v>0.10463215258855582</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>70</v>
@@ -4996,7 +4992,7 @@
       </c>
       <c r="B14" s="4">
         <f>COUNTIF(WBS!U5:U137,"Complete")</f>
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>72</v>
@@ -6244,7 +6240,7 @@
         <v>0</v>
       </c>
       <c r="Q18" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R18" s="14">
         <f t="shared" si="0"/>
@@ -6256,11 +6252,11 @@
       </c>
       <c r="T18" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U18" t="str">
         <f>IF(Q18&gt;=1,"Complete",IF(Q18&gt;0,"In Progress",IF(Control!$B$7&lt;H18,"Not Started",IF(Control!$B$7&gt;I18,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V18" s="15">
         <v>46265</v>
@@ -6317,7 +6313,7 @@
         <v>0</v>
       </c>
       <c r="Q19" s="14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R19" s="14">
         <f t="shared" si="0"/>
@@ -6329,11 +6325,11 @@
       </c>
       <c r="T19" s="17">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>5.4495912806539499E-3</v>
       </c>
       <c r="U19" t="str">
         <f>IF(Q19&gt;=1,"Complete",IF(Q19&gt;0,"In Progress",IF(Control!$B$7&lt;H19,"Not Started",IF(Control!$B$7&gt;I19,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>Complete</v>
       </c>
       <c r="V19" s="15">
         <v>46272</v>
@@ -15318,22 +15314,22 @@
       </c>
       <c r="H8" s="6">
         <f>IFERROR(SUMIF(WBS!$D$5:$D$137,A8,WBS!$T$5:$T$137)/SUMIF(WBS!$D$5:$D$137,A8,WBS!$R$5:$R$137),0)</f>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I8" s="6">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="J8" s="4">
         <v>3</v>
       </c>
       <c r="K8" s="4">
         <f>COUNTIFS(WBS!$D$5:$D$137,A8,WBS!$U$5:$U$137,"Complete")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L8" s="4" t="str">
         <f>IF(H8&gt;=1,"Complete",IF(H8&gt;0,"In Progress",IF(Control!$B$7&lt;D8,"Not Started",IF(Control!$B$7&gt;E8,"Late","Ready"))))</f>
-        <v>Not Started</v>
+        <v>In Progress</v>
       </c>
     </row>
     <row r="9" spans="1:12">
@@ -16973,7 +16969,7 @@
       </c>
       <c r="I4" s="6">
         <f>IF(A4=Control!$B$7,Control!$B$11,"")</f>
-        <v>0.10463215258855582</v>
+        <v>0.11553133514986372</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="42.75">

</xml_diff>